<commit_message>
bugfix: rm spaces in column names
</commit_message>
<xml_diff>
--- a/tests/broadcast.xlsx
+++ b/tests/broadcast.xlsx
@@ -25,31 +25,31 @@
     <t xml:space="preserve">org_id</t>
   </si>
   <si>
-    <t xml:space="preserve"> org_name</t>
+    <t xml:space="preserve">org_name</t>
   </si>
   <si>
     <t xml:space="preserve">region_id</t>
   </si>
   <si>
-    <t xml:space="preserve"> smi_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> smi_rating</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> smi_male_proportion</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> district_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> district_population</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> frequency</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> power</t>
+    <t xml:space="preserve">smi_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">smi_rating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">smi_male_proportion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">district_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">district_population</t>
+  </si>
+  <si>
+    <t xml:space="preserve">frequency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">power</t>
   </si>
   <si>
     <t xml:space="preserve">Тест</t>

</xml_diff>